<commit_message>
Batch 1: move Sign out into a gear account menu
- Gear icon now opens a dropdown (name/email + role, Settings link, Sign out)
  that closes on outside click; removed the standalone logout icon.
- Module switcher unchanged (already lists accessible modules + closes on blur).
- Verified: tsc 0, build clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Status.xlsx
+++ b/Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude\YeldnIN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB7E8332-5502-403B-A4CC-1F8AC6A36D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B88423-5EE6-41DD-9045-A23318578D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{03BFBFE4-6B78-43D9-97D2-4634F79151D7}"/>
   </bookViews>
@@ -39,20 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
-  <si>
-    <t>Request</t>
-  </si>
-  <si>
-    <t>Order</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
   <si>
     <t>Sales</t>
   </si>
   <si>
-    <t>Dispatch</t>
-  </si>
-  <si>
     <t>Trip</t>
   </si>
   <si>
@@ -77,9 +68,6 @@
     <t>New</t>
   </si>
   <si>
-    <t xml:space="preserve">New </t>
-  </si>
-  <si>
     <t>Transit</t>
   </si>
   <si>
@@ -99,6 +87,99 @@
   </si>
   <si>
     <t>Dispatched</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Started Shipping</t>
+  </si>
+  <si>
+    <t>Completed Shipping</t>
+  </si>
+  <si>
+    <t>Purchasing</t>
+  </si>
+  <si>
+    <t>In Egypt</t>
+  </si>
+  <si>
+    <t>Ready to pickup</t>
+  </si>
+  <si>
+    <t>Picked up</t>
+  </si>
+  <si>
+    <t>Transfer</t>
+  </si>
+  <si>
+    <t>Purchase</t>
+  </si>
+  <si>
+    <t>Patch</t>
+  </si>
+  <si>
+    <t>Shipment</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>After 2 or 4 days (randomly) of being received by hub or trip, item status changes automatically to Transit</t>
+  </si>
+  <si>
+    <t>After 4 or 6 days (randomly) of being received by hub or trip, item status changes automatically to Global Shipping</t>
+  </si>
+  <si>
+    <t>Requested</t>
+  </si>
+  <si>
+    <t>New Request placed by sales including that item</t>
+  </si>
+  <si>
+    <t>Item was purchased by purchasing team</t>
+  </si>
+  <si>
+    <t>Item put in dispatch, or purchased status changed to dispatched</t>
+  </si>
+  <si>
+    <t>Purchase or Patch marked delivered</t>
+  </si>
+  <si>
+    <t>Purchase or Patch marked received</t>
+  </si>
+  <si>
+    <t>When Trip status change to In Egypt, Item Status change to Customs</t>
+  </si>
+  <si>
+    <t>When Trip status change to (Ready to pickup), Item Status change to (Out for Delivery)</t>
+  </si>
+  <si>
+    <t>When Trip or shipment status change to (Picked up), Item Status change to (Office)</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Logistics</t>
+  </si>
+  <si>
+    <t>Delivered to hub</t>
+  </si>
+  <si>
+    <t>Received by hub</t>
+  </si>
+  <si>
+    <t>Shipped to destination</t>
+  </si>
+  <si>
+    <t>Delivered to destination</t>
+  </si>
+  <si>
+    <t>Received in destination</t>
+  </si>
+  <si>
+    <t>Left Origin</t>
   </si>
 </sst>
 </file>
@@ -140,9 +221,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,117 +567,265 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6176B5CD-F41E-4E97-BF04-8EED21822C69}">
-  <dimension ref="B4:F17"/>
+  <dimension ref="A2:P19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="45.453125" customWidth="1"/>
     <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="L3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G7" t="s">
+        <v>18</v>
+      </c>
+      <c r="P7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8" t="s">
+        <v>43</v>
+      </c>
+      <c r="P8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
         <v>3</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
       </c>
-      <c r="D9" t="s">
+      <c r="L9" t="s">
+        <v>44</v>
+      </c>
+      <c r="P9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" t="s">
+        <v>45</v>
+      </c>
+      <c r="P10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
+    <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+      <c r="G17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
+      <c r="G18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
-        <v>18</v>
+      <c r="G19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:G2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(integration): match inbound customers by email (cross-store dedup)
The customer sync matched only on veeeyCustomerId (a per-store account id).
veeey.com already populated it on every YeldnIN customer, so a veeey.net
push — different ids, same real people — would have created ~16k duplicates.

Now Customer carries a normalized email, and handleCustomerUpsert matches
EMAIL first (the identity shared by the same person across both stores),
then veeeyCustomerId, then name. On match it re-keys veeeyCustomerId to the
inbound id — veeey.net is the main store now, so it becomes the identity
owner (owner-approved).

Migration adds Customer.email + index. parseWireCustomer lowercases the
incoming email. All 478 tests pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Status.xlsx
+++ b/Status.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude\YeldnIN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B88423-5EE6-41DD-9045-A23318578D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CFD892-CE8A-4B01-9AD0-EFFE38173575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{03BFBFE4-6B78-43D9-97D2-4634F79151D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,8 +39,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={F6CED279-1A1B-4C8D-8852-D65574633730}</author>
+  </authors>
+  <commentList>
+    <comment ref="I17" authorId="0" shapeId="0" xr:uid="{F6CED279-1A1B-4C8D-8852-D65574633730}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    System will generate new shipments as soon as the trip is approved (OK) by admins</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="50">
   <si>
     <t>Sales</t>
   </si>
@@ -122,9 +141,6 @@
     <t>Shipment</t>
   </si>
   <si>
-    <t>Item</t>
-  </si>
-  <si>
     <t>After 2 or 4 days (randomly) of being received by hub or trip, item status changes automatically to Transit</t>
   </si>
   <si>
@@ -180,19 +196,37 @@
   </si>
   <si>
     <t>Left Origin</t>
+  </si>
+  <si>
+    <t>Special Order Item</t>
+  </si>
+  <si>
+    <t>Out of Stock/ Restock / Optional Item</t>
+  </si>
+  <si>
+    <t>When Operation staff send photos of the pickup shipment to Sales team through the system</t>
+  </si>
+  <si>
+    <t>When Sales mark shipment as (Website)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -225,13 +259,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -248,6 +282,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Mohamed Abotaleb" id="{DFF6CC6B-66EF-4863-8B3E-0B9E76251B68}" userId="7db542731dad2dbb" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -565,266 +605,343 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="I17" dT="2026-06-16T08:24:19.63" personId="{DFF6CC6B-66EF-4863-8B3E-0B9E76251B68}" id="{F6CED279-1A1B-4C8D-8852-D65574633730}">
+    <text>System will generate new shipments as soon as the trip is approved (OK) by admins</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6176B5CD-F41E-4E97-BF04-8EED21822C69}">
-  <dimension ref="A2:P19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6176B5CD-F41E-4E97-BF04-8EED21822C69}">
+  <dimension ref="A2:J19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="45.453125" customWidth="1"/>
     <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.26953125" customWidth="1"/>
+    <col min="4" max="5" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="G4" t="s">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="G5" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H5" t="s">
         <v>16</v>
       </c>
-      <c r="L5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="G6" t="s">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H6" t="s">
         <v>17</v>
       </c>
-      <c r="L6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="G7" t="s">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H7" t="s">
         <v>18</v>
       </c>
-      <c r="P7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>31</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="L8" t="s">
-        <v>43</v>
-      </c>
-      <c r="P8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>32</v>
       </c>
       <c r="B9" t="s">
         <v>3</v>
       </c>
       <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
         <v>8</v>
       </c>
-      <c r="L9" t="s">
-        <v>44</v>
-      </c>
-      <c r="P9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>33</v>
+    </row>
+    <row r="10" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D10" t="s">
         <v>15</v>
       </c>
-      <c r="L10" t="s">
-        <v>45</v>
-      </c>
-      <c r="P10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
       <c r="D11" t="s">
         <v>5</v>
       </c>
       <c r="E11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="F11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
       </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
       <c r="D12" t="s">
         <v>6</v>
       </c>
       <c r="E12" t="s">
         <v>6</v>
       </c>
-      <c r="G12" t="s">
+      <c r="F12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>28</v>
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>29</v>
+    <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>37</v>
+    <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
       </c>
-      <c r="G16" t="s">
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" t="s">
         <v>21</v>
       </c>
-      <c r="H16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
-        <v>38</v>
+    </row>
+    <row r="17" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="B17" t="s">
         <v>2</v>
       </c>
-      <c r="G17" t="s">
-        <v>22</v>
+      <c r="C17" t="s">
+        <v>2</v>
       </c>
       <c r="H17" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="B18" t="s">
         <v>13</v>
       </c>
-      <c r="G18" t="s">
+      <c r="C18" t="s">
         <v>13</v>
       </c>
       <c r="H18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="B19" t="s">
         <v>14</v>
       </c>
-      <c r="G19" t="s">
+      <c r="C19" t="s">
         <v>14</v>
       </c>
       <c r="H19" t="s">
         <v>14</v>
       </c>
+      <c r="I19" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:G2"/>
+  <mergeCells count="3">
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64DB4E00-DBB2-4235-9992-1E732A236914}">
+  <dimension ref="B2:C10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="3" width="20.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>